<commit_message>
IPO Desk: SFC Environmental Technologies rebuilt from the RHP
RHP dated 19-Oct-2026 (FY26 financials, offer terms, dates, peers).
Call Subscribe at the Rs 330 upper band; fair value Rs 358 / 392 / 423;
reported P/E 20.9x, adjusted 21.2x.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sh3XfYSpHMqTXgPXQV3Xds
</commit_message>
<xml_diff>
--- a/ipo-analysis/companies/sfc-environmental-technologies-ltd/SFC_ENVIRONMENTAL_TECHNO_01_Screening.xlsx
+++ b/ipo-analysis/companies/sfc-environmental-technologies-ltd/SFC_ENVIRONMENTAL_TECHNO_01_Screening.xlsx
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr"/>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>45894</v>
+        <v>46314</v>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
     </row>
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>45747</v>
+        <v>46203</v>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>none (all figures from the DRHP and its corrigendum)</t>
+          <t>Price band and lot size from the NSE issue page</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
@@ -1307,17 +1307,20 @@
         </is>
       </c>
       <c r="C5" s="16" t="n">
-        <v>519.447</v>
+        <v>657.495</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>657.495</v>
+        <v>697.8579999999999</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>697.8579999999999</v>
+        <v>803.629</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>133.944</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>p. 364</t>
+          <t>p. 412</t>
         </is>
       </c>
     </row>
@@ -1328,17 +1331,20 @@
         </is>
       </c>
       <c r="C6" s="16" t="n">
-        <v>11.378</v>
+        <v>19.071</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>19.071</v>
+        <v>29.106</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>29.106</v>
+        <v>17.643</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>3.952</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>pp. 364, 422</t>
+          <t>pp. 412, 471</t>
         </is>
       </c>
     </row>
@@ -1349,17 +1355,20 @@
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>127.251</v>
+        <v>193.447</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>193.447</v>
+        <v>205.239</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>205.239</v>
+        <v>211.488</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>2.151</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>p. 364</t>
+          <t>p. 412</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1379,20 @@
         </is>
       </c>
       <c r="C8" s="16" t="n">
-        <v>33.224</v>
+        <v>50.546</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>50.546</v>
+        <v>53.499</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>53.499</v>
+        <v>56.64</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>1.891</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>p. 364</t>
+          <t>p. 412</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1403,20 @@
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>-0.782</v>
+        <v>-1.273</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>-1.273</v>
+        <v>-0.268</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>-0.268</v>
+        <v>-5.365</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>-1.224</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>p. 364 (deferred tax plus MAT credit)</t>
+          <t>p. 412 (deferred tax plus MAT credit)</t>
         </is>
       </c>
     </row>
@@ -1412,17 +1427,20 @@
         </is>
       </c>
       <c r="C10" s="16" t="n">
-        <v>93.881</v>
+        <v>141.607</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>141.607</v>
+        <v>144.06</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>144.06</v>
+        <v>154.361</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>1.511</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>p. 364 (attributable to owners; total PAT Rs 94.81 / 144.17 / 152.01 cr)</t>
+          <t>p. 412 (attributable to owners; total PAT Rs 144.17 / 152.01 / 160.21 cr)</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1451,20 @@
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>30.391</v>
+        <v>-11.694</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>-11.694</v>
+        <v>65.509</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>65.509</v>
+        <v>-25.802</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>-21.342</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>p. 368</t>
+          <t>p. 417</t>
         </is>
       </c>
     </row>
@@ -1454,17 +1475,20 @@
         </is>
       </c>
       <c r="C12" s="16" t="n">
-        <v>6.68</v>
+        <v>0.408</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.39</v>
+        <v>0.018</v>
       </c>
       <c r="E12" s="16" t="n">
         <v>0.018</v>
       </c>
+      <c r="F12" s="16" t="n">
+        <v>0.005</v>
+      </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>pp. 34-35 (HWTPL services before it became a subsidiary; Turbomax rent)</t>
+          <t>pp. 99-100</t>
         </is>
       </c>
     </row>
@@ -1475,17 +1499,20 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>0</v>
+        <v>1.578</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>1.578</v>
+        <v>3.281</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>pp. 34-35 (Turbomax purchases and services; reimbursements)</t>
+          <t>pp. 99-100 (Turbomax India purchases and services)</t>
         </is>
       </c>
     </row>
@@ -1496,17 +1523,20 @@
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>395.416</v>
+        <v>534.296</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>534.296</v>
+        <v>648.682</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>648.682</v>
+        <v>804.173</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>805.4880000000001</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>p. 362 (owners)</t>
+          <t>p. 411 (owners)</t>
         </is>
       </c>
     </row>
@@ -1517,17 +1547,20 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>238.238</v>
+        <v>394.514</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>394.514</v>
+        <v>487.371</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>487.371</v>
+        <v>660.172</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>511.112</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>pp. 362, 406-409 (current + non-current)</t>
+          <t>p. 411 (current + non-current)</t>
         </is>
       </c>
     </row>
@@ -1538,17 +1571,20 @@
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>73.80800000000001</v>
+        <v>108.408</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>108.408</v>
+        <v>97.583</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>97.583</v>
+        <v>125.14</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>142.3</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>p. 362</t>
+          <t>p. 411</t>
         </is>
       </c>
     </row>
@@ -1559,17 +1595,20 @@
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>107.772</v>
+        <v>110.714</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>110.714</v>
+        <v>93.17</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>93.17</v>
+        <v>170.268</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>75.15000000000001</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>p. 363</t>
+          <t>p. 411</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1619,7 @@
         </is>
       </c>
       <c r="C18" s="16" t="n">
-        <v>0.45</v>
+        <v>0.021</v>
       </c>
       <c r="D18" s="16" t="n">
         <v>0.021</v>
@@ -1588,9 +1627,12 @@
       <c r="E18" s="16" t="n">
         <v>0.021</v>
       </c>
+      <c r="F18" s="16" t="n">
+        <v>0.021</v>
+      </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>p. 34</t>
+          <t>p. 98</t>
         </is>
       </c>
     </row>
@@ -1607,11 +1649,14 @@
         <v>2.808</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>2.808</v>
+        <v>30.322</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>30.322</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>p. 362</t>
+          <t>pp. 411, 457</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1686,7 @@
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>0.1676</v>
+        <v>0.1434</v>
       </c>
     </row>
     <row r="24">
@@ -1651,7 +1696,7 @@
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>0.6137</v>
+        <v>0.6444</v>
       </c>
     </row>
     <row r="25">
@@ -1661,7 +1706,7 @@
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>0.1034</v>
+        <v>0.1718</v>
       </c>
     </row>
     <row r="26">
@@ -1697,7 +1742,7 @@
         </is>
       </c>
       <c r="E29" s="16" t="n">
-        <v>150</v>
+        <v>667.53</v>
       </c>
     </row>
     <row r="31">
@@ -2358,12 +2403,12 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>pp. 43-46, 119</t>
+          <t>pp. 186, 412</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
         <is>
-          <t>1:5 split (05-Sep-2024) and 2:1 bonus (05-Sep-2024) are reflected: EPS 10.05 / 15.16 / 15.42 FY23-25 are on the post-bonus count of 9,34,11,270 shares.</t>
+          <t>9,34,11,270 shares of Rs 2 (post 1:5 split and 2:1 bonus of Sep-2024); FY26 EPS Rs 16.52. No pre-IPO placement was made; share count unchanged since the DRHP.</t>
         </is>
       </c>
     </row>
@@ -2395,12 +2440,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>pp. 34, 368</t>
+          <t>pp. 188, 417</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>Operating cash flow Rs 30.39 cr / -11.69 cr / 65.51 cr FY23-25 against PAT Rs 94.81 / 144.17 / 152.01 cr: cumulative CFO/PAT about 22% (owners' PAT basis). Working capital rose from 27.8% to 63.5% of revenue as receivable days went 158 -&gt; 197 -&gt; 262. FY25 cash flow recovered as collections improved; typical of a technology supplier paid on municipal STP project milestones, but the trend is the key thing to track.</t>
+          <t>Operating cash flow Rs -11.69 / +65.51 / -25.80 cr FY24-26 against owners' PAT Rs 141.61 / 144.06 / 154.36 cr: cumulative CFO 6% of PAT. Trade receivables rose by Rs 173.64 cr in FY26; cash conversion cycle 156 -&gt; 232 -&gt; 242 days (411 days at Jun-26, seasonal). Q1 FY27 CFO -Rs 21.34 cr. The working-capital object (Rs 74.92 cr) is sized for this.</t>
         </is>
       </c>
     </row>
@@ -2432,12 +2477,12 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>pp. 364, 368</t>
+          <t>pp. 412, 417</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>Current tax 26.1% of cumulative FY23-25 PBT; income tax paid Rs 135.80 cr over three years. Profit is taxed in cash.</t>
+          <t>Current tax 27.0% of FY26 PBT; income tax paid Rs 60.00 cr in FY26. Profit is taxed in cash.</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2514,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>pp. 34-36</t>
+          <t>pp. 99-100</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
-          <t>Related-party dealings outside the group are small (Turbomax India purchases Rs 1.58 cr FY25). Large intra-group loans to SWT subsidiaries (Vasudha, HWTPL, Pentagen) are eliminated on consolidation. Dividends Rs 31.14 cr paid in FY25.</t>
+          <t>Related-party dealings outside the group are small (Turbomax India purchases Rs 3.28 cr in FY26; Rs 12.25 cr equity investment in Turbomax). CMD pay Rs 4.21 cr in FY26. Interim dividend of Rs 28.02 cr (Rs 3 a share) declared 04-Sep-2026, before the IPO.</t>
         </is>
       </c>
     </row>
@@ -2506,12 +2551,12 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>pp. 151-152</t>
+          <t>p. 168</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>Fresh issue is amount-based (Rs 150 cr), no fixed share count. Rs 47.46 cr repays debt (company and Vasudha Waste Treatment), Rs 69.67 cr funds working capital, balance GCP (cap 25%) and expenses. No capex object.</t>
+          <t>Amount-based fresh issue (Rs 150 cr): Rs 42.23 cr debt prepayment, Rs 74.92 cr working capital (both in FY27), balance GCP. No capex object, no fixed share count.</t>
         </is>
       </c>
     </row>
@@ -2567,17 +2612,17 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>pp. 362, 402</t>
+          <t>pp. 457, 510</t>
         </is>
       </c>
       <c r="G11" s="27" t="inlineStr">
         <is>
-          <t>Goodwill Rs 2.81 cr; other intangibles Rs 7.26 cr are service-concession rights acquired with a subsidiary in Oct-2023, amortised Rs 5.57 cr a year - not capitalised development costs.</t>
+          <t>Goodwill up from Rs 2.81 cr to Rs 30.32 cr after buying 80% of IST-Anlagenbau GmbH (Germany, solar sludge dryers) on 30-Jul-2025 for Rs 32.32 cr, against Rs 4.81 cr of net assets acquired; no impairment so far.</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2654,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>pp. 48, 54</t>
+          <t>pp. 48, 307</t>
         </is>
       </c>
       <c r="G12" s="27" t="inlineStr">
         <is>
-          <t>Top customer 16.76% and top-10 61.37% of FY25 revenue (EPC contractors building municipal STPs); top-10 suppliers 47.71% of purchases. Usual for a project-linked technology supplier.</t>
+          <t>Top customer 14.34% and top-10 64.44% of FY26 revenue (79.20% in the seasonal Q1 FY27); top supplier 17.18% of purchases.</t>
         </is>
       </c>
     </row>
@@ -2646,12 +2691,12 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>pp. 33, 508</t>
+          <t>pp. 554-557</t>
         </is>
       </c>
       <c r="G13" s="27" t="inlineStr">
         <is>
-          <t>Contingent liabilities tiny (Rs 0.02 cr), but subsidiary SFC Umwelttechnik GmbH faces a EUR 5.60 m (Rs 56.75 cr, 8.7% of FY25 net worth) liquidated-damages suit in Portugal over a 2018 STP supply; defence filed 28-Oct-2024, pending.</t>
+          <t>Ten show-cause notices (Jul-2025 to Sep-2026) from the Goa SPCB and GWMC to subsidiaries HWTPL and VWTPL over effluent and waste-handling at the North and South Goa plants, plus the Aug-2025 FIR; responses filed, all pending. Portugal claim EUR 5.60 m (Rs 59.75 cr, 7.4% of net worth) against SFC Umwelttechnik GmbH pending; two ex-MDs of that subsidiary claim about EUR 0.2-0.3 m in Austria.</t>
         </is>
       </c>
     </row>
@@ -2716,12 +2761,12 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>pp. 356-358</t>
+          <t>p. 403</t>
         </is>
       </c>
       <c r="G15" s="27" t="inlineStr">
         <is>
-          <t>G B C A &amp; Associates LLP audit with no qualifications; two overseas subsidiaries (FY25 assets Rs 23.02 cr, revenue Rs 20.07 cr) are consolidated on unaudited, management-certified accounts. Small, but should be audited by the RHP.</t>
+          <t>G B C A &amp; Associates LLP; no qualifications. Overseas subsidiaries' accounts partly certified by management (FY24-25 per DRHP); confirm audit status in the RHP auditor's report.</t>
         </is>
       </c>
     </row>
@@ -2782,12 +2827,12 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>p. 151</t>
+          <t>p. 168</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
         <is>
-          <t>Fresh issue Rs 150 cr: a monitoring agency is mandatory above Rs 50 cr; to be named in the RHP.</t>
+          <t>Fresh issue Rs 150 cr: monitoring agency required.</t>
         </is>
       </c>
     </row>
@@ -2880,17 +2925,17 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>p. 529</t>
+          <t>pp. 575-578</t>
         </is>
       </c>
       <c r="G20" s="27" t="inlineStr">
         <is>
-          <t>BRLMs IIFL Capital, JM Financial and Nuvama: IIFL and JM track records are in the desk database; Nuvama not yet compiled.</t>
+          <t>IIFL Capital and JM Financial track records in the desk database; Nuvama's FY27 issues listed in the RHP.</t>
         </is>
       </c>
     </row>
@@ -2917,19 +2962,11 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>N.A.</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>p. 151</t>
-        </is>
-      </c>
-      <c r="G21" s="27" t="inlineStr">
-        <is>
-          <t>No capex object.</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="27" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E21">

</xml_diff>